<commit_message>
chore: updated portfolio mockups and added hover badges
</commit_message>
<xml_diff>
--- a/SocialMedia.xlsx
+++ b/SocialMedia.xlsx
@@ -323,10 +323,12 @@
     <t>Vê como transformámos a marca X</t>
   </si>
   <si>
-    <t>Exemplo de texto PT sobre: Novo Projeto Lançado</t>
-  </si>
-  <si>
-    <t>EN text example about: Novo Projeto Lançado</t>
+    <t xml:space="preserve">O design tem o poder de reposicionar uma marca no mercado. Neste novo projeto, fomos ao detalhe para criar uma experiência digital que reflete a verdadeira essência e ambição do nosso cliente. Desde a arquitetura de informação à interface, cada elemento foi pensado para guiar o utilizador de forma fluida e impactante. Curioso para ver o resultado final e os bastidores deste desafio de crescimento e visibilidade?
+Clica no link e vê o portfólio.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Design has the power to reposition a brand in the market. In this new project, we went down to the details to create a digital experience that reflects the true essence and ambition of our client. From information architecture to the interface, every element was designed to guide the user in a fluid and impactful way. Curious to see the final result and the scenes behind this B2B growth and visibility challenge?
+Click the link and see the portfolio.</t>
   </si>
   <si>
     <t>https://sueste.com/</t>
@@ -362,10 +364,12 @@
     <t>Estás a perder clientes se o teu site tem isto</t>
   </si>
   <si>
-    <t>Exemplo de texto PT sobre: 3 erros no design do site</t>
-  </si>
-  <si>
-    <t>EN text example about: 3 erros no design do site</t>
+    <t xml:space="preserve">Um site não pode ser apenas bonito, tem de converter. Na nossa experiência a analisar presenças digitais B2B, estes são os 3 erros que mais afastam potenciais clientes: mensagens confusas, navegação pouco intuitiva e falta de apelos à ação claros. Estes atritos destroem a confiança de quem tenta perceber como podes ajudar. Queres parar de perder oportunidades através do teu site?
+Vamos conversar. Entra no link e pede um orçamento para reestruturarmos a tua presença digital.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A website can't just be beautiful, it has to convert. In our experience analyzing B2B digital presences, these are the 3 mistakes that most drive potential clients away: confusing messaging, unintuitive navigation, and a lack of clear calls to action. These frictions destroy the trust of anyone trying to understand how you can help. Want to stop losing opportunities through your website?
+Let's talk. Enter the link and request a quote to restructure your digital presence.</t>
   </si>
   <si>
     <t>Reunião de brainstorm</t>
@@ -374,10 +378,12 @@
     <t>Espreita como nascem as ideias</t>
   </si>
   <si>
-    <t>Exemplo de texto PT sobre: Reunião de brainstorm</t>
-  </si>
-  <si>
-    <t>EN text example about: Reunião de brainstorm</t>
+    <t xml:space="preserve">Antes da primeira linha de código ou mockup, o trabalho começa aqui. Quando nos desafiam a resolver um obstáculo de crescimento, sentamo-nos à mesa com um objetivo claro: encontrar um ângulo diferenciador que alinhe estratégia com criatividade. Os primeiros rascunhos são sempre caóticos, mas é do caos focado que sugem as melhores soluções digitais. Qual é o vosso processo favorito para arrancar novos projetos?
+Acede ao nosso link para saberes mais sobre como trabalhamos.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Before the first line of code or mockup, the work begins right here. When challenged to solve a growth obstacle, we sit around the table with one clear goal: to find a differentiating angle that aligns strategy with creativity. The first drafts are always chaotic, but it is from focused chaos that the best digital solutions emerge. What is your favorite process to kick off new projects?
+Access our link to know more about how we work.</t>
   </si>
   <si>
     <t>social_w2</t>
@@ -389,10 +395,12 @@
     <t>Precisa de um site novo este mês?</t>
   </si>
   <si>
-    <t>Exemplo de texto PT sobre: Pacote Criação Websites</t>
-  </si>
-  <si>
-    <t>EN text example about: Pacote Criação Websites</t>
+    <t xml:space="preserve">Dar um salto na visibilidade do teu negócio não precisa de demorar meses. O nosso pacote de criação de websites foi desenhado especificamente para empresas B2B que querem avançar rapidamente mantendo uma imagem premium focada em conversão. Estruturamos a proposta de valor, desenhamos a interface à medida e entregamos um site pronto para impulsionar resultados.
+Pronto para o próximo passo? Usa o link e contacta-nos.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Taking a leap in your business visibility doesn't need to take months. Our website creation package is tailored specifically for B2B companies looking to move quickly while maintaining a premium image focused on conversion. We structure your value proposition, design a custom interface, and deliver a website ready to boost results.
+Ready for the next step? Use the link and contact us.</t>
   </si>
   <si>
     <t>O que dizem de nós</t>
@@ -401,10 +409,12 @@
     <t>"A Sueste mudou o nosso negócio"</t>
   </si>
   <si>
-    <t>Exemplo de texto PT sobre: O que dizem de nós</t>
-  </si>
-  <si>
-    <t>EN text example about: O que dizem de nós</t>
+    <t xml:space="preserve">O final de um projeto web só é um sucesso quando o cliente vê mudanças reais no dia a dia. Ouvir que a nova plataforma melhorou métricas cruciais é o maior reconhecimento da eficácia do nosso método. Mais do que estética, a nossa agência foca-se em entregar ferramentas digitais sólidas que posicionam a marca como líder no seu mercado.
+Queres ver o que temos construído? Vai ao link e vê o nosso portfólio completo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The end of a web project is only a success when the client sees real changes day-to-day. Hearing that the new platform improved crucial metrics is the greatest acknowledgment of our method's effectiveness. More than aesthetics, our agency focuses on delivering solid digital tools that position the brand as a leader in its market.
+Want to see what we've been building? Go to the link and see our complete portfolio.</t>
   </si>
   <si>
     <t>social_w3</t>
@@ -416,10 +426,12 @@
     <t>Hoje a equipa da Sueste esteve focada em...</t>
   </si>
   <si>
-    <t>Exemplo de texto PT sobre: 1 dia no nosso escritório</t>
-  </si>
-  <si>
-    <t>EN text example about: 1 dia no nosso escritório</t>
+    <t xml:space="preserve">Um dia de trabalho na Sueste nunca é igual ao anterior. Hoje a prioridade foi refinar a arquitetura de informação de uma plataforma B2B, focar em sessões de UX/UI, e garantir a performance mobile. O segredo de um projeto coeso está no trabalho de equipa e na constante otimização.
+Queres saber mais sobre e conhecer quem faz a magia acontecer? Clica no link e descobre.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">A workday at Sueste is never the same as the last. Today, the priority was refining the information architecture of a B2B platform, focusing on UX/UI sessions, and ensuring mobile performance. The secret to a cohesive project lies in teamwork and constant optimization.
+Want to know more and meet who makes the magic happen? Click the link and discover.</t>
   </si>
   <si>
     <t>Aumento de 200% tráfego</t>
@@ -428,10 +440,12 @@
     <t>Como fizemos o site Y crescer 200%</t>
   </si>
   <si>
-    <t>Exemplo de texto PT sobre: Aumento de 200% tráfego</t>
-  </si>
-  <si>
-    <t>EN text example about: Aumento de 200% tráfego</t>
+    <t xml:space="preserve">Dados que falam mais alto do que promessas. Quando assumimos este caso de estudo, o diagnóstico inicial revelou fortes falhas na retenção. Aplicámos metodologias de UX focadas em acessibilidade e reposicionámos o copy da landing page. O resultado? Um crescimento de 200% no tráfego qualificado que aumentou a geração de leads do cliente num mercado altamente competitivo.
+Clica no link e explora como o fizemos neste novo artigo.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Data that speaks louder than promises. When we took on this case study, the initial diagnosis revealed strong flaws in retention. We applied UX methodologies focused on accessibility and repositioned the landing page's copy. The result? A 200% growth in qualified traffic that increased the client's lead generation in a highly competitive market.
+Click the link and explore how we did it in this new article.</t>
   </si>
   <si>
     <t>social_w4</t>
@@ -1700,7 +1714,7 @@
         <v>46082</v>
       </c>
       <c r="V2" t="s">
-        <v>33</v>
+        <v>43</v>
       </c>
       <c r="W2" t="s">
         <v>106</v>
@@ -1783,7 +1797,7 @@
         <v>46085</v>
       </c>
       <c r="V3" t="s">
-        <v>33</v>
+        <v>43</v>
       </c>
       <c r="W3" t="s">
         <v>106</v>
@@ -1866,7 +1880,7 @@
         <v>46089</v>
       </c>
       <c r="V4" t="s">
-        <v>33</v>
+        <v>43</v>
       </c>
       <c r="W4" t="s">
         <v>106</v>
@@ -1949,7 +1963,7 @@
         <v>46092</v>
       </c>
       <c r="V5" t="s">
-        <v>33</v>
+        <v>43</v>
       </c>
       <c r="W5" t="s">
         <v>106</v>
@@ -2032,7 +2046,7 @@
         <v>46096</v>
       </c>
       <c r="V6" t="s">
-        <v>33</v>
+        <v>43</v>
       </c>
       <c r="W6" t="s">
         <v>106</v>
@@ -2115,7 +2129,7 @@
         <v>46099</v>
       </c>
       <c r="V7" t="s">
-        <v>33</v>
+        <v>43</v>
       </c>
       <c r="W7" t="s">
         <v>106</v>
@@ -2198,7 +2212,7 @@
         <v>46103</v>
       </c>
       <c r="V8" t="s">
-        <v>33</v>
+        <v>43</v>
       </c>
       <c r="W8" t="s">
         <v>106</v>
@@ -2281,7 +2295,7 @@
         <v>46106</v>
       </c>
       <c r="V9" t="s">
-        <v>33</v>
+        <v>43</v>
       </c>
       <c r="W9" t="s">
         <v>106</v>
@@ -2364,7 +2378,7 @@
         <v>46110</v>
       </c>
       <c r="V10" t="s">
-        <v>33</v>
+        <v>43</v>
       </c>
       <c r="W10" t="s">
         <v>106</v>
@@ -2447,7 +2461,7 @@
         <v>46112.95833333333</v>
       </c>
       <c r="V11" t="s">
-        <v>33</v>
+        <v>43</v>
       </c>
       <c r="W11" t="s">
         <v>106</v>
@@ -2530,7 +2544,7 @@
         <v>46116.95833333333</v>
       </c>
       <c r="V12" t="s">
-        <v>33</v>
+        <v>43</v>
       </c>
       <c r="W12" t="s">
         <v>106</v>
@@ -2613,7 +2627,7 @@
         <v>46119.95833333333</v>
       </c>
       <c r="V13" t="s">
-        <v>33</v>
+        <v>43</v>
       </c>
       <c r="W13" t="s">
         <v>106</v>
@@ -2696,7 +2710,7 @@
         <v>46123.95833333333</v>
       </c>
       <c r="V14" t="s">
-        <v>33</v>
+        <v>43</v>
       </c>
       <c r="W14" t="s">
         <v>106</v>
@@ -2779,7 +2793,7 @@
         <v>46126.95833333333</v>
       </c>
       <c r="V15" t="s">
-        <v>33</v>
+        <v>43</v>
       </c>
       <c r="W15" t="s">
         <v>106</v>
@@ -2862,7 +2876,7 @@
         <v>46130.95833333333</v>
       </c>
       <c r="V16" t="s">
-        <v>33</v>
+        <v>43</v>
       </c>
       <c r="W16" t="s">
         <v>106</v>
@@ -2945,7 +2959,7 @@
         <v>46133.95833333333</v>
       </c>
       <c r="V17" t="s">
-        <v>33</v>
+        <v>43</v>
       </c>
       <c r="W17" t="s">
         <v>106</v>
@@ -3028,7 +3042,7 @@
         <v>46137.95833333333</v>
       </c>
       <c r="V18" t="s">
-        <v>33</v>
+        <v>43</v>
       </c>
       <c r="W18" t="s">
         <v>106</v>
@@ -3111,7 +3125,7 @@
         <v>46140.95833333333</v>
       </c>
       <c r="V19" t="s">
-        <v>33</v>
+        <v>43</v>
       </c>
       <c r="W19" t="s">
         <v>106</v>
@@ -3194,7 +3208,7 @@
         <v>46144.95833333333</v>
       </c>
       <c r="V20" t="s">
-        <v>33</v>
+        <v>43</v>
       </c>
       <c r="W20" t="s">
         <v>106</v>
@@ -3277,7 +3291,7 @@
         <v>46147.95833333333</v>
       </c>
       <c r="V21" t="s">
-        <v>33</v>
+        <v>43</v>
       </c>
       <c r="W21" t="s">
         <v>106</v>
@@ -3360,7 +3374,7 @@
         <v>46151.95833333333</v>
       </c>
       <c r="V22" t="s">
-        <v>33</v>
+        <v>43</v>
       </c>
       <c r="W22" t="s">
         <v>106</v>
@@ -3443,7 +3457,7 @@
         <v>46154.95833333333</v>
       </c>
       <c r="V23" t="s">
-        <v>33</v>
+        <v>43</v>
       </c>
       <c r="W23" t="s">
         <v>106</v>
@@ -3526,7 +3540,7 @@
         <v>46158.95833333333</v>
       </c>
       <c r="V24" t="s">
-        <v>33</v>
+        <v>43</v>
       </c>
       <c r="W24" t="s">
         <v>106</v>
@@ -3609,7 +3623,7 @@
         <v>46161.95833333333</v>
       </c>
       <c r="V25" t="s">
-        <v>33</v>
+        <v>43</v>
       </c>
       <c r="W25" t="s">
         <v>106</v>

</xml_diff>